<commit_message>
Added new data source in xslx and txt
</commit_message>
<xml_diff>
--- a/src/Case/TNO_data_Erasmus_case.xlsx
+++ b/src/Case/TNO_data_Erasmus_case.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365tno-my.sharepoint.com/personal/siemen_nooren_tno_nl/Documents/Documents/2025/Erasmus/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malonekm\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="8_{2EFE8F21-7443-4CFD-8E43-82EC8C9009F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D22DDFE4-2285-4843-8581-3B0BF8435E92}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12CA9F5A-5B73-4F0A-AD50-F65CC165CF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{13B18F91-3E73-4336-96C7-077297EB6E52}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{13B18F91-3E73-4336-96C7-077297EB6E52}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="59">
   <si>
     <t>Assumptions:</t>
   </si>
@@ -55,143 +55,173 @@
     <t>Each truck can perform at most one delivery per day</t>
   </si>
   <si>
+    <t>The scenario lasts for 10 days.</t>
+  </si>
+  <si>
+    <t>The figure to the right represents the FD concept. Each supply centre is assigned a number of operating units or other supply centres. It has to ensure that they do not experience a stockout. The arrows indicate for which operating units or other supply centres a supply centre is reponsible for.</t>
+  </si>
+  <si>
+    <t>Daily usage in kg</t>
+  </si>
+  <si>
+    <t>Maximum storage capacity in kg</t>
+  </si>
+  <si>
+    <t>Order information</t>
+  </si>
+  <si>
+    <t>Operating unit</t>
+  </si>
+  <si>
+    <t>Food&amp;water</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Ammunition</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Order time</t>
+  </si>
+  <si>
+    <t>Time Window</t>
+  </si>
+  <si>
+    <t>Driving time to source in seconds</t>
+  </si>
+  <si>
+    <t>Vust</t>
+  </si>
+  <si>
+    <t>MSC</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
+    <t>22:00-00:00</t>
+  </si>
+  <si>
+    <t>Sample a value from a uniform distribution with parameters (minimum = 0.8, maximum = 1.2), then multiply this sampled value by the daily usage for each day and each operating unit.</t>
+  </si>
+  <si>
+    <t>Sample a value from a binomial distribution with parameters (number of trials = 25, probability of success = 0.4), then multiply this sampled value by the daily usage and divide it by 10 for each day and each operating unit.</t>
+  </si>
+  <si>
+    <t>Gn cie 1</t>
+  </si>
+  <si>
+    <t>FSC 1</t>
+  </si>
+  <si>
+    <t>16:00</t>
+  </si>
+  <si>
+    <t>20:00-02:00</t>
+  </si>
+  <si>
+    <t>Gn cie 2</t>
+  </si>
+  <si>
+    <t>FSC 2</t>
+  </si>
+  <si>
+    <t>Painf cie 1</t>
+  </si>
+  <si>
+    <t>Painf cie 2</t>
+  </si>
+  <si>
+    <t>Painf cie 3</t>
+  </si>
+  <si>
+    <t>Painf cie 4</t>
+  </si>
+  <si>
+    <t>Painf cie 5</t>
+  </si>
+  <si>
+    <t>AT cie 1</t>
+  </si>
+  <si>
+    <t>AT cie 2</t>
+  </si>
+  <si>
+    <t>AT cie 3</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>CCLs content in kg</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Type 1</t>
+  </si>
+  <si>
+    <t>Type 2</t>
+  </si>
+  <si>
+    <t>Type 3</t>
+  </si>
+  <si>
+    <t>Stochastic usage</t>
+  </si>
+  <si>
+    <t>ß</t>
+  </si>
+  <si>
+    <t>Sample a value from a triangular distribution with parameters (minimum = 0.2, mode = 0.8, maximum = 2.0), then multiply this sampled value by the daily usage for each day and each operating unit.</t>
+  </si>
+  <si>
+    <t>Trucks belong to a warehouse and cannot be reassigned or reallocated</t>
+  </si>
+  <si>
+    <t>Storage of warehouses is given in data tab</t>
+  </si>
+  <si>
+    <t>Maximum storage capacity (in CCLs)</t>
+  </si>
+  <si>
+    <t>Initial storage levels</t>
+  </si>
+  <si>
+    <t>Gn cie</t>
+  </si>
+  <si>
+    <t>Painf cie</t>
+  </si>
+  <si>
+    <t>AT cie</t>
+  </si>
+  <si>
+    <t>CCL type 1</t>
+  </si>
+  <si>
+    <t>CCL type 2</t>
+  </si>
+  <si>
+    <t>CCL Type 3</t>
+  </si>
+  <si>
+    <t>Can can only drive downstream one level and back: In the FD concept, this means: MSC-FSC; FSC-OU;MSC-Vust</t>
+  </si>
+  <si>
     <t>Storage of warehouses and operating units is full at the start.</t>
-  </si>
-  <si>
-    <t>The scenario lasts for 10 days.</t>
-  </si>
-  <si>
-    <t>The figure to the right represents the FD concept. Each supply centre is assigned a number of operating units or other supply centres. It has to ensure that they do not experience a stockout. The arrows indicate for which operating units or other supply centres a supply centre is reponsible for.</t>
-  </si>
-  <si>
-    <t>Daily usage in kg</t>
-  </si>
-  <si>
-    <t>Maximum storage capacity in kg</t>
-  </si>
-  <si>
-    <t>Order information</t>
-  </si>
-  <si>
-    <t>Operating unit</t>
-  </si>
-  <si>
-    <t>Food&amp;water</t>
-  </si>
-  <si>
-    <t>Fuel</t>
-  </si>
-  <si>
-    <t>Ammunition</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Order time</t>
-  </si>
-  <si>
-    <t>Time Window</t>
-  </si>
-  <si>
-    <t>Driving time to source in seconds</t>
-  </si>
-  <si>
-    <t>Vust</t>
-  </si>
-  <si>
-    <t>MSC</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>22:00-00:00</t>
-  </si>
-  <si>
-    <t>Sample a value from a uniform distribution with parameters (minimum = 0.8, maximum = 1.2), then multiply this sampled value by the daily usage for each day and each operating unit.</t>
-  </si>
-  <si>
-    <t>Sample a value from a binomial distribution with parameters (number of trials = 25, probability of success = 0.4), then multiply this sampled value by the daily usage and divide it by 10 for each day and each operating unit.</t>
-  </si>
-  <si>
-    <t>Gn cie 1</t>
-  </si>
-  <si>
-    <t>FSC 1</t>
-  </si>
-  <si>
-    <t>16:00</t>
-  </si>
-  <si>
-    <t>20:00-02:00</t>
-  </si>
-  <si>
-    <t>Gn cie 2</t>
-  </si>
-  <si>
-    <t>FSC 2</t>
-  </si>
-  <si>
-    <t>Painf cie 1</t>
-  </si>
-  <si>
-    <t>Painf cie 2</t>
-  </si>
-  <si>
-    <t>Painf cie 3</t>
-  </si>
-  <si>
-    <t>Painf cie 4</t>
-  </si>
-  <si>
-    <t>Painf cie 5</t>
-  </si>
-  <si>
-    <t>AT cie 1</t>
-  </si>
-  <si>
-    <t>AT cie 2</t>
-  </si>
-  <si>
-    <t>AT cie 3</t>
-  </si>
-  <si>
-    <t>infinity</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>CCLs content in kg</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Type 1</t>
-  </si>
-  <si>
-    <t>Type 2</t>
-  </si>
-  <si>
-    <t>Type 3</t>
-  </si>
-  <si>
-    <t>Stochastic usage</t>
-  </si>
-  <si>
-    <t>ß</t>
-  </si>
-  <si>
-    <t>Sample a value from a triangular distribution with parameters (minimum = 0.2, mode = 0.8, maximum = 2.0), then multiply this sampled value by the daily usage for each day and each operating unit.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -203,6 +233,19 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -228,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -243,11 +286,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -637,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21002443-C020-4805-BCB9-EA4C3F308302}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="98.5703125" customWidth="1"/>
@@ -669,17 +738,29 @@
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
+      <c r="A6" s="17" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -696,7 +777,7 @@
   <sheetData>
     <row r="2" spans="1:1" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -707,7 +788,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75D4CC89-EBFD-4297-8ADC-9B6CAB8E55F7}">
-  <dimension ref="B2:R42"/>
+  <dimension ref="B2:U42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -723,75 +804,75 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" t="s">
+        <v>11</v>
+      </c>
+      <c r="N3" t="s">
         <v>12</v>
       </c>
-      <c r="G3" t="s">
+      <c r="O3" t="s">
         <v>13</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" t="s">
-        <v>17</v>
-      </c>
-      <c r="L3" t="s">
-        <v>18</v>
-      </c>
-      <c r="M3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N3" t="s">
-        <v>13</v>
-      </c>
-      <c r="O3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4">
         <v>13018</v>
@@ -812,30 +893,30 @@
         <v>201420</v>
       </c>
       <c r="I4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" t="s">
         <v>20</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>21</v>
-      </c>
-      <c r="K4" t="s">
-        <v>22</v>
       </c>
       <c r="L4">
         <v>3997</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="M4" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="N4" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>48</v>
+      <c r="O4" s="16" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5">
         <v>6209</v>
@@ -856,24 +937,24 @@
         <v>131154</v>
       </c>
       <c r="I5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" t="s">
         <v>26</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>27</v>
-      </c>
-      <c r="K5" t="s">
-        <v>28</v>
       </c>
       <c r="L5">
         <v>17611</v>
       </c>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6">
         <v>6966</v>
@@ -894,24 +975,24 @@
         <v>118428</v>
       </c>
       <c r="I6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" t="s">
         <v>27</v>
-      </c>
-      <c r="K6" t="s">
-        <v>28</v>
       </c>
       <c r="L6">
         <v>17824</v>
       </c>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7">
         <v>8086</v>
@@ -932,24 +1013,24 @@
         <v>174666</v>
       </c>
       <c r="I7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" t="s">
         <v>26</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>27</v>
-      </c>
-      <c r="K7" t="s">
-        <v>28</v>
       </c>
       <c r="L7">
         <v>15904</v>
       </c>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8">
         <v>11197</v>
@@ -970,24 +1051,24 @@
         <v>182028</v>
       </c>
       <c r="I8" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" t="s">
         <v>26</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>27</v>
-      </c>
-      <c r="K8" t="s">
-        <v>28</v>
       </c>
       <c r="L8">
         <v>14911</v>
       </c>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C9">
         <v>9447</v>
@@ -1008,24 +1089,24 @@
         <v>172512</v>
       </c>
       <c r="I9" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" t="s">
         <v>26</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>27</v>
-      </c>
-      <c r="K9" t="s">
-        <v>28</v>
       </c>
       <c r="L9">
         <v>17587</v>
       </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C10">
         <v>11570</v>
@@ -1046,24 +1127,24 @@
         <v>158832</v>
       </c>
       <c r="I10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K10" t="s">
         <v>27</v>
-      </c>
-      <c r="K10" t="s">
-        <v>28</v>
       </c>
       <c r="L10">
         <v>18385</v>
       </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11">
         <v>10351</v>
@@ -1084,24 +1165,24 @@
         <v>167544</v>
       </c>
       <c r="I11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J11" t="s">
+        <v>26</v>
+      </c>
+      <c r="K11" t="s">
         <v>27</v>
-      </c>
-      <c r="K11" t="s">
-        <v>28</v>
       </c>
       <c r="L11">
         <v>17169</v>
       </c>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12">
         <v>3476</v>
@@ -1122,24 +1203,24 @@
         <v>52809</v>
       </c>
       <c r="I12" t="s">
+        <v>25</v>
+      </c>
+      <c r="J12" t="s">
         <v>26</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>27</v>
-      </c>
-      <c r="K12" t="s">
-        <v>28</v>
       </c>
       <c r="L12">
         <v>15547</v>
       </c>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="16"/>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C13">
         <v>2484</v>
@@ -1160,24 +1241,24 @@
         <v>55854</v>
       </c>
       <c r="I13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J13" t="s">
         <v>26</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>27</v>
-      </c>
-      <c r="K13" t="s">
-        <v>28</v>
       </c>
       <c r="L13">
         <v>14078</v>
       </c>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="16"/>
+      <c r="O13" s="16"/>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14">
         <v>3033</v>
@@ -1198,62 +1279,90 @@
         <v>49017</v>
       </c>
       <c r="I14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J14" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" t="s">
         <v>27</v>
-      </c>
-      <c r="K14" t="s">
-        <v>28</v>
       </c>
       <c r="L14">
         <v>15071</v>
       </c>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C17" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6" t="s">
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="16"/>
+    </row>
+    <row r="17" spans="2:21" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="H17" s="10"/>
+      <c r="I17" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+      <c r="P17" s="13"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="13"/>
+      <c r="S17" s="13"/>
+      <c r="T17" s="13"/>
+      <c r="U17" s="13"/>
+    </row>
+    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
         <v>12</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>13</v>
       </c>
-      <c r="E18" t="s">
+      <c r="I18" t="s">
         <v>14</v>
       </c>
-      <c r="F18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" t="s">
-        <v>14</v>
-      </c>
-      <c r="I18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="J18" t="s">
+        <v>15</v>
+      </c>
+      <c r="K18" t="s">
+        <v>16</v>
+      </c>
+      <c r="L18" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="T18" s="14"/>
+      <c r="U18" s="14"/>
+    </row>
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1264,22 +1373,49 @@
       <c r="E19">
         <v>0</v>
       </c>
-      <c r="F19" t="s">
-        <v>39</v>
-      </c>
-      <c r="G19" t="s">
-        <v>39</v>
-      </c>
-      <c r="H19" t="s">
-        <v>39</v>
-      </c>
       <c r="I19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="J19" t="s">
+        <v>38</v>
+      </c>
+      <c r="K19" t="s">
+        <v>38</v>
+      </c>
+      <c r="L19" t="s">
+        <v>38</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q19" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="R19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="T19" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="U19" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1290,23 +1426,54 @@
       <c r="E20">
         <v>0</v>
       </c>
-      <c r="F20">
-        <v>132237</v>
-      </c>
-      <c r="G20">
-        <v>384717</v>
-      </c>
-      <c r="H20">
-        <v>752049</v>
-      </c>
-      <c r="I20">
-        <v>18334</v>
-      </c>
-      <c r="O20" s="5"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="F20" s="6">
+        <v>126</v>
+      </c>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J20" s="7">
+        <v>0.75</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L20" s="6">
+        <v>21934</v>
+      </c>
+      <c r="M20" s="6">
+        <v>7</v>
+      </c>
+      <c r="N20" s="6">
+        <v>7</v>
+      </c>
+      <c r="O20" s="11">
+        <v>7</v>
+      </c>
+      <c r="P20" s="6">
+        <v>29</v>
+      </c>
+      <c r="Q20" s="6">
+        <v>29</v>
+      </c>
+      <c r="R20" s="6">
+        <v>29</v>
+      </c>
+      <c r="S20" s="6">
+        <v>6</v>
+      </c>
+      <c r="T20" s="6">
+        <v>6</v>
+      </c>
+      <c r="U20" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1317,50 +1484,81 @@
       <c r="E21">
         <v>0</v>
       </c>
-      <c r="F21">
-        <v>89991</v>
-      </c>
-      <c r="G21">
-        <v>244344</v>
-      </c>
-      <c r="H21">
-        <v>553665</v>
-      </c>
-      <c r="I21">
-        <v>18665</v>
-      </c>
-      <c r="O21" s="5"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="F21" s="6">
+        <v>87</v>
+      </c>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J21" s="7">
+        <v>0.75</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" s="6">
+        <v>22165</v>
+      </c>
+      <c r="M21" s="6">
+        <v>7</v>
+      </c>
+      <c r="N21" s="6">
+        <v>7</v>
+      </c>
+      <c r="O21" s="11">
+        <v>7</v>
+      </c>
+      <c r="P21" s="6">
+        <v>19</v>
+      </c>
+      <c r="Q21" s="6">
+        <v>19</v>
+      </c>
+      <c r="R21" s="6">
+        <v>19</v>
+      </c>
+      <c r="S21" s="6">
+        <v>3</v>
+      </c>
+      <c r="T21" s="6">
+        <v>3</v>
+      </c>
+      <c r="U21" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
       <c r="O22" s="5"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
       <c r="O23" s="5"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
+        <v>39</v>
+      </c>
+      <c r="O24" s="5"/>
+    </row>
+    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="O25" s="5"/>
+    </row>
+    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
         <v>41</v>
-      </c>
-      <c r="O24" s="5"/>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25" t="s">
-        <v>14</v>
-      </c>
-      <c r="O25" s="5"/>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>43</v>
       </c>
       <c r="C26">
         <v>3000</v>
@@ -1373,9 +1571,9 @@
       </c>
       <c r="O26" s="5"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C27">
         <v>1000</v>
@@ -1388,9 +1586,9 @@
       </c>
       <c r="O27" s="5"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -1403,10 +1601,10 @@
       </c>
       <c r="O28" s="5"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
       <c r="O29" s="5"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
       <c r="O30" s="5"/>
     </row>
     <row r="34" spans="13:18" x14ac:dyDescent="0.25">
@@ -1414,7 +1612,7 @@
     </row>
     <row r="37" spans="13:18" x14ac:dyDescent="0.25">
       <c r="R37" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="13:18" x14ac:dyDescent="0.25">
@@ -1424,16 +1622,20 @@
       <c r="M42" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="13">
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="I17:L17"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="M4:M14"/>
     <mergeCell ref="N4:N14"/>
     <mergeCell ref="O4:O14"/>
-    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="M17:U17"/>
+    <mergeCell ref="M18:O18"/>
+    <mergeCell ref="P18:R18"/>
+    <mergeCell ref="S18:U18"/>
     <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="I2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>